<commit_message>
refactor: remove price deletion example script and update template spreadsheets
</commit_message>
<xml_diff>
--- a/public/templates/Planilla_de_eliminacion_de_precios_por_SKU.xlsx
+++ b/public/templates/Planilla_de_eliminacion_de_precios_por_SKU.xlsx
@@ -26,14 +26,14 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="00F8FAFC"/>
       <sz val="11"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
-      <sz val="10"/>
+      <name val="Calibri"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -45,8 +45,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E11D48"/>
-        <bgColor rgb="00E11D48"/>
+        <fgColor rgb="001E293B"/>
+        <bgColor rgb="001E293B"/>
       </patternFill>
     </fill>
   </fills>
@@ -60,29 +60,32 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00E2E8F0"/>
       </left>
       <right style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00E2E8F0"/>
       </right>
       <top style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00E2E8F0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00CBD5E1"/>
+        <color rgb="00E2E8F0"/>
       </bottom>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -452,11 +455,11 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>SKU ID</t>
@@ -468,31 +471,31 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+        <v>1001</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t>cyber</t>
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+        <v>1002</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t>organizacion</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+        <v>1003</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>test</t>
         </is>

</xml_diff>